<commit_message>
feat(ui): stream temporal display — all series as columns in bottom panel
- selecting an item shows ALL its time series in ONE bottom table: a year row
  index with one editable column per temporal attribute (price, sale_price, …)
- removed the redundant per-item nested '↳ attr · by year' rail subitems; temporal
  datasets are reached by selecting the item (→ bottom) or via the 'Temporal
  datasets' group at the foot of the left rail

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/pathwise/public/examples/steel.xlsx
+++ b/frontend/pathwise/public/examples/steel.xlsx
@@ -1626,7 +1626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1642,20 +1642,15 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>group</t>
+          <t>baseline_technology</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>baseline_technology</t>
+          <t>capacity</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
-        <is>
-          <t>capacity</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
         <is>
           <t>introduced_year</t>
         </is>
@@ -1669,23 +1664,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pohang BF3</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
           <t>BF-BOF</t>
         </is>
       </c>
+      <c r="D2" t="n">
+        <v>4128000</v>
+      </c>
       <c r="E2" t="n">
-        <v>4128000</v>
-      </c>
-      <c r="F2" t="n">
         <v>2017</v>
       </c>
     </row>
@@ -1697,23 +1687,18 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HyundaiBF3</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hyundai Steel</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
           <t>BF-BOF</t>
         </is>
       </c>
+      <c r="D3" t="n">
+        <v>4000000</v>
+      </c>
       <c r="E3" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="F3" t="n">
         <v>2013</v>
       </c>
     </row>
@@ -1725,23 +1710,18 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pohang BF4</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
           <t>BF-BOF</t>
         </is>
       </c>
+      <c r="D4" t="n">
+        <v>3804000</v>
+      </c>
       <c r="E4" t="n">
-        <v>3804000</v>
-      </c>
-      <c r="F4" t="n">
         <v>2024</v>
       </c>
     </row>
@@ -1753,23 +1733,18 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Gwangyang BF2</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
           <t>BF-BOF</t>
         </is>
       </c>
+      <c r="D5" t="n">
+        <v>3239000</v>
+      </c>
       <c r="E5" t="n">
-        <v>3239000</v>
-      </c>
-      <c r="F5" t="n">
         <v>2006</v>
       </c>
     </row>
@@ -1781,23 +1756,18 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gwangyang BF1</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
           <t>BF-BOF</t>
         </is>
       </c>
+      <c r="D6" t="n">
+        <v>1683000</v>
+      </c>
       <c r="E6" t="n">
-        <v>1683000</v>
-      </c>
-      <c r="F6" t="n">
         <v>2013</v>
       </c>
     </row>
@@ -1809,23 +1779,18 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gwangyang BF5</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
           <t>BF-BOF</t>
         </is>
       </c>
+      <c r="D7" t="n">
+        <v>4722000</v>
+      </c>
       <c r="E7" t="n">
-        <v>4722000</v>
-      </c>
-      <c r="F7" t="n">
         <v>2016</v>
       </c>
     </row>
@@ -1837,23 +1802,18 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HyundaiBF2</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hyundai Steel</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
           <t>BF-BOF</t>
         </is>
       </c>
+      <c r="D8" t="n">
+        <v>4237000</v>
+      </c>
       <c r="E8" t="n">
-        <v>4237000</v>
-      </c>
-      <c r="F8" t="n">
         <v>2010</v>
       </c>
     </row>
@@ -1865,23 +1825,18 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gwangyang BF4</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
           <t>BF-BOF</t>
         </is>
       </c>
+      <c r="D9" t="n">
+        <v>4000000</v>
+      </c>
       <c r="E9" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="F9" t="n">
         <v>2022</v>
       </c>
     </row>
@@ -1893,23 +1848,18 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Gwangyang BF3</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
           <t>BF-BOF</t>
         </is>
       </c>
+      <c r="D10" t="n">
+        <v>3624000</v>
+      </c>
       <c r="E10" t="n">
-        <v>3624000</v>
-      </c>
-      <c r="F10" t="n">
         <v>2020</v>
       </c>
     </row>
@@ -1921,23 +1871,18 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HyundaiBF1</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hyundai Steel</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
           <t>BF-BOF</t>
         </is>
       </c>
+      <c r="D11" t="n">
+        <v>4127000</v>
+      </c>
       <c r="E11" t="n">
-        <v>4127000</v>
-      </c>
-      <c r="F11" t="n">
         <v>2010</v>
       </c>
     </row>
@@ -1949,23 +1894,18 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pohang BF2</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
           <t>BF-BOF</t>
         </is>
       </c>
+      <c r="D12" t="n">
+        <v>4000000</v>
+      </c>
       <c r="E12" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="F12" t="n">
         <v>2015</v>
       </c>
     </row>
@@ -1977,23 +1917,18 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Pohang FNX3</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
           <t>BF-BOF-FX</t>
         </is>
       </c>
+      <c r="D13" t="n">
+        <v>1914000</v>
+      </c>
       <c r="E13" t="n">
-        <v>1914000</v>
-      </c>
-      <c r="F13" t="n">
         <v>2015</v>
       </c>
     </row>
@@ -2005,23 +1940,18 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pohang FNX2</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
           <t>BF-BOF-FX</t>
         </is>
       </c>
+      <c r="D14" t="n">
+        <v>1280000</v>
+      </c>
       <c r="E14" t="n">
-        <v>1280000</v>
-      </c>
-      <c r="F14" t="n">
         <v>2015</v>
       </c>
     </row>
@@ -2033,23 +1963,18 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EAF1</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
           <t>EAF</t>
         </is>
       </c>
+      <c r="D15" t="n">
+        <v>2500000</v>
+      </c>
       <c r="E15" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="F15" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -2061,23 +1986,18 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EAF2</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
           <t>EAF</t>
         </is>
       </c>
+      <c r="D16" t="n">
+        <v>2500000</v>
+      </c>
       <c r="E16" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="F16" t="n">
         <v>2027</v>
       </c>
     </row>
@@ -2089,23 +2009,18 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EAF3</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
           <t>EAF</t>
         </is>
       </c>
+      <c r="D17" t="n">
+        <v>1000000</v>
+      </c>
       <c r="E17" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="F17" t="n">
         <v>2029</v>
       </c>
     </row>
@@ -2120,7 +2035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2148,7 +2063,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pohang BF3</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2160,13 +2075,13 @@
         <v>2025</v>
       </c>
       <c r="D2" t="n">
-        <v>4128000</v>
+        <v>32394000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pohang BF3</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2178,13 +2093,13 @@
         <v>2030</v>
       </c>
       <c r="D3" t="n">
-        <v>3574624</v>
+        <v>34051447</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pohang BF3</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2196,13 +2111,13 @@
         <v>2035</v>
       </c>
       <c r="D4" t="n">
-        <v>3574624</v>
+        <v>34051447</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pohang BF3</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2214,13 +2129,13 @@
         <v>2040</v>
       </c>
       <c r="D5" t="n">
-        <v>3574624</v>
+        <v>34051447</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pohang BF3</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2232,13 +2147,13 @@
         <v>2045</v>
       </c>
       <c r="D6" t="n">
-        <v>3574624</v>
+        <v>34051447</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pohang BF3</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2250,13 +2165,13 @@
         <v>2050</v>
       </c>
       <c r="D7" t="n">
-        <v>3574624</v>
+        <v>34051447</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HyundaiBF3</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2268,13 +2183,13 @@
         <v>2025</v>
       </c>
       <c r="D8" t="n">
-        <v>4000000</v>
+        <v>12364000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HyundaiBF3</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2286,13 +2201,13 @@
         <v>2030</v>
       </c>
       <c r="D9" t="n">
-        <v>3463783</v>
+        <v>10706553</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HyundaiBF3</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2304,13 +2219,13 @@
         <v>2035</v>
       </c>
       <c r="D10" t="n">
-        <v>3463783</v>
+        <v>10706553</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HyundaiBF3</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2322,13 +2237,13 @@
         <v>2040</v>
       </c>
       <c r="D11" t="n">
-        <v>3463783</v>
+        <v>10706553</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HyundaiBF3</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2340,13 +2255,13 @@
         <v>2045</v>
       </c>
       <c r="D12" t="n">
-        <v>3463783</v>
+        <v>10706553</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HyundaiBF3</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2358,1519 +2273,7 @@
         <v>2050</v>
       </c>
       <c r="D13" t="n">
-        <v>3463783</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Pohang BF4</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D14" t="n">
-        <v>3804000</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Pohang BF4</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D15" t="n">
-        <v>3294058</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Pohang BF4</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D16" t="n">
-        <v>3294058</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Pohang BF4</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D17" t="n">
-        <v>3294058</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Pohang BF4</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D18" t="n">
-        <v>3294058</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Pohang BF4</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D19" t="n">
-        <v>3294058</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Gwangyang BF2</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D20" t="n">
-        <v>3239000</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Gwangyang BF2</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D21" t="n">
-        <v>2804798</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Gwangyang BF2</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D22" t="n">
-        <v>2804798</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Gwangyang BF2</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D23" t="n">
-        <v>2804798</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Gwangyang BF2</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D24" t="n">
-        <v>2804798</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Gwangyang BF2</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D25" t="n">
-        <v>2804798</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Gwangyang BF1</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D26" t="n">
-        <v>1683000</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Gwangyang BF1</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D27" t="n">
-        <v>1457387</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Gwangyang BF1</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D28" t="n">
-        <v>1457387</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Gwangyang BF1</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D29" t="n">
-        <v>1457387</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Gwangyang BF1</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D30" t="n">
-        <v>1457387</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Gwangyang BF1</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D31" t="n">
-        <v>1457387</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Gwangyang BF5</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D32" t="n">
-        <v>4722000</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Gwangyang BF5</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D33" t="n">
-        <v>4088996</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Gwangyang BF5</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D34" t="n">
-        <v>4088996</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Gwangyang BF5</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D35" t="n">
-        <v>4088996</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Gwangyang BF5</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D36" t="n">
-        <v>4088996</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Gwangyang BF5</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D37" t="n">
-        <v>4088996</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>HyundaiBF2</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D38" t="n">
-        <v>4237000</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>HyundaiBF2</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D39" t="n">
-        <v>3669012</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>HyundaiBF2</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D40" t="n">
-        <v>3669012</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>HyundaiBF2</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D41" t="n">
-        <v>3669012</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>HyundaiBF2</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D42" t="n">
-        <v>3669012</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>HyundaiBF2</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D43" t="n">
-        <v>3669012</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Gwangyang BF4</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D44" t="n">
-        <v>4000000</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Gwangyang BF4</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D45" t="n">
-        <v>3463783</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Gwangyang BF4</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D46" t="n">
-        <v>3463783</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Gwangyang BF4</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D47" t="n">
-        <v>3463783</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Gwangyang BF4</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D48" t="n">
-        <v>3463783</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Gwangyang BF4</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D49" t="n">
-        <v>3463783</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Gwangyang BF3</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D50" t="n">
-        <v>3624000</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Gwangyang BF3</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D51" t="n">
-        <v>3138187</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Gwangyang BF3</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D52" t="n">
-        <v>3138187</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Gwangyang BF3</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D53" t="n">
-        <v>3138187</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Gwangyang BF3</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D54" t="n">
-        <v>3138187</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Gwangyang BF3</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D55" t="n">
-        <v>3138187</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>HyundaiBF1</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D56" t="n">
-        <v>4127000</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>HyundaiBF1</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D57" t="n">
-        <v>3573758</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>HyundaiBF1</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D58" t="n">
-        <v>3573758</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>HyundaiBF1</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C59" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D59" t="n">
-        <v>3573758</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>HyundaiBF1</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D60" t="n">
-        <v>3573758</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>HyundaiBF1</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D61" t="n">
-        <v>3573758</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Pohang BF2</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D62" t="n">
-        <v>4000000</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Pohang BF2</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D63" t="n">
-        <v>3463783</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Pohang BF2</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D64" t="n">
-        <v>3463783</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Pohang BF2</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D65" t="n">
-        <v>3463783</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Pohang BF2</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D66" t="n">
-        <v>3463783</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Pohang BF2</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D67" t="n">
-        <v>3463783</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Pohang FNX3</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D68" t="n">
-        <v>1914000</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Pohang FNX3</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C69" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D69" t="n">
-        <v>1657420</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Pohang FNX3</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C70" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D70" t="n">
-        <v>1657420</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Pohang FNX3</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C71" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D71" t="n">
-        <v>1657420</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Pohang FNX3</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C72" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D72" t="n">
-        <v>1657420</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Pohang FNX3</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C73" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D73" t="n">
-        <v>1657420</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Pohang FNX2</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C74" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D74" t="n">
-        <v>1280000</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Pohang FNX2</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C75" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D75" t="n">
-        <v>1108411</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Pohang FNX2</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C76" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D76" t="n">
-        <v>1108411</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Pohang FNX2</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C77" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D77" t="n">
-        <v>1108411</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Pohang FNX2</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C78" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D78" t="n">
-        <v>1108411</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Pohang FNX2</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C79" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D79" t="n">
-        <v>1108411</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>EAF1</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C80" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D80" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>EAF1</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C81" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D81" t="n">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>EAF1</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C82" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D82" t="n">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>EAF1</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C83" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D83" t="n">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>EAF1</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C84" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D84" t="n">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>EAF1</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C85" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D85" t="n">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>EAF2</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C86" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D86" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>EAF2</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C87" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D87" t="n">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>EAF2</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C88" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D88" t="n">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>EAF2</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C89" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D89" t="n">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>EAF2</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C90" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D90" t="n">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>EAF2</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C91" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D91" t="n">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>EAF3</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C92" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D92" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>EAF3</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C93" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D93" t="n">
-        <v>1000000</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>EAF3</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C94" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D94" t="n">
-        <v>1000000</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>EAF3</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C95" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D95" t="n">
-        <v>1000000</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>EAF3</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C96" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D96" t="n">
-        <v>1000000</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>EAF3</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C97" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D97" t="n">
-        <v>1000000</v>
+        <v>10706553</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(data): steel as a 2-stage iron-making → steel-making chain
Each integrated route is decomposed into iron-making (fuels + iron-ore → iron)
and steel-making (iron + scrap → steel), linked by a 1:1 'iron' intermediate via
routing edges — so the route's per-tonne inputs/emissions/costs are preserved
exactly while the chain becomes visible (Simple view shows iron facilities above
steel facilities). Iron decarbonises BF→H2-DRI; steel BOF→ESF/EAF. EAF stays
single-stage (scrap→steel). 29 facilities, 7 techs; solves optimal.

steel.py carries the source-based 2-stage converter; the shipped steel.xlsx was
regenerated by an in-place transform (source xlsx currently unavailable). Fuel
intensity = fuel per unit production (GJ/t, MWh, GJ/km) = the io coefficient.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/pathwise/public/examples/steel.xlsx
+++ b/frontend/pathwise/public/examples/steel.xlsx
@@ -19,10 +19,11 @@
     <sheet name="technologies_t__opex" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="technologies_t__renewal" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="io" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="processes" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="demand" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="transitions" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="impact_caps" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="edges" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="processes" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="demand" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="transitions" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="impact_caps" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,7 +452,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Steel (Korea, PLANiT MACC)</t>
+          <t>Steel (Korea, PLANiT MACC) — iron→steel chain</t>
         </is>
       </c>
     </row>
@@ -476,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,20 +488,35 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>BOF</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
+          <t>BF-FX</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
+        <is>
+          <t>BOF-FX</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>H2-DRI</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ESF</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>EAF</t>
         </is>
@@ -511,15 +527,24 @@
         <v>2025</v>
       </c>
       <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
         <v>250350</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
         <v>212797.5</v>
       </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
         <v>550000</v>
       </c>
-      <c r="E2" t="n">
+      <c r="H2" t="n">
         <v>120000</v>
       </c>
     </row>
@@ -528,15 +553,24 @@
         <v>2030</v>
       </c>
       <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
         <v>250350</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
         <v>212797.5</v>
       </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
         <v>550000</v>
       </c>
-      <c r="E3" t="n">
+      <c r="H3" t="n">
         <v>120000</v>
       </c>
     </row>
@@ -545,15 +579,24 @@
         <v>2035</v>
       </c>
       <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
         <v>250350</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
         <v>212797.5</v>
       </c>
-      <c r="D4" t="n">
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
         <v>550000</v>
       </c>
-      <c r="E4" t="n">
+      <c r="H4" t="n">
         <v>120000</v>
       </c>
     </row>
@@ -562,15 +605,24 @@
         <v>2040</v>
       </c>
       <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
         <v>250350</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
         <v>212797.5</v>
       </c>
-      <c r="D5" t="n">
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
         <v>550000</v>
       </c>
-      <c r="E5" t="n">
+      <c r="H5" t="n">
         <v>120000</v>
       </c>
     </row>
@@ -579,15 +631,24 @@
         <v>2045</v>
       </c>
       <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
         <v>250350</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
         <v>212797.5</v>
       </c>
-      <c r="D6" t="n">
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
         <v>550000</v>
       </c>
-      <c r="E6" t="n">
+      <c r="H6" t="n">
         <v>120000</v>
       </c>
     </row>
@@ -596,15 +657,24 @@
         <v>2050</v>
       </c>
       <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
         <v>250350</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>212797.5</v>
       </c>
-      <c r="D7" t="n">
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
         <v>550000</v>
       </c>
-      <c r="E7" t="n">
+      <c r="H7" t="n">
         <v>120000</v>
       </c>
     </row>
@@ -619,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -630,20 +700,35 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>BOF</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
+          <t>BF-FX</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
+        <is>
+          <t>BOF-FX</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>H2-DRI</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ESF</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>EAF</t>
         </is>
@@ -657,12 +742,21 @@
         <v>200280</v>
       </c>
       <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
         <v>170238</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
         <v>440000</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
         <v>96000</v>
       </c>
     </row>
@@ -674,12 +768,21 @@
         <v>200280</v>
       </c>
       <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
         <v>170238</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
         <v>440000</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
         <v>96000</v>
       </c>
     </row>
@@ -691,12 +794,21 @@
         <v>200280</v>
       </c>
       <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
         <v>170238</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
         <v>440000</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
         <v>96000</v>
       </c>
     </row>
@@ -708,12 +820,21 @@
         <v>200280</v>
       </c>
       <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
         <v>170238</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
         <v>440000</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
         <v>96000</v>
       </c>
     </row>
@@ -725,12 +846,21 @@
         <v>200280</v>
       </c>
       <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
         <v>170238</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
         <v>440000</v>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
         <v>96000</v>
       </c>
     </row>
@@ -742,12 +872,21 @@
         <v>200280</v>
       </c>
       <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
         <v>170238</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
         <v>440000</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>96000</v>
       </c>
     </row>
@@ -762,7 +901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -810,7 +949,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -842,7 +981,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -874,7 +1013,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -906,7 +1045,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -938,7 +1077,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -970,7 +1109,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1002,7 +1141,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1020,7 +1159,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>feedstock</t>
+          <t>feed_ore</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -1034,44 +1173,36 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Scrap_BB</t>
+          <t>iron</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>input</t>
+          <t>output</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>feedstock</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.3</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BOF</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HBI_BB</t>
+          <t>iron</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1080,56 +1211,54 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>feedstock</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.3</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BOF</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>Scrap_BB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>output</t>
+          <t>input</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="b">
-        <v>1</v>
-      </c>
+        <v>0.11</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>feed_scrap</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>BOF</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Coal_BX</t>
+          <t>HBI_BB</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1138,62 +1267,56 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>15.054042</v>
+        <v>0</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>fuel</t>
+          <t>feed_scrap</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>BOF</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BF gas_BX</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>input</t>
+          <t>output</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1.90404</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>fuel</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H13" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>BF-FX</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BOF gas_BX</t>
+          <t>Coal_BX</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1202,7 +1325,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.21156</v>
+        <v>15.054042</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1210,22 +1333,22 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>BF-FX</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Natural gas_BX</t>
+          <t>BF gas_BX</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1234,7 +1357,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.48092</v>
+        <v>1.90404</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1252,12 +1375,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>BF-FX</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Iron ore_BX</t>
+          <t>BOF gas_BX</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1266,56 +1389,62 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1.65</v>
+        <v>0.21156</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>feedstock</t>
+          <t>fuel</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>BF-FX</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>Natural gas_BX</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>output</t>
+          <t>input</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="b">
-        <v>1</v>
-      </c>
+        <v>1.48092</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>fuel</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
+          <t>BF-FX</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Hydrogen_H2</t>
+          <t>Iron ore_BX</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1324,62 +1453,54 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>9.395454545454545</v>
+        <v>1.65</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>fuel</t>
+          <t>feed_ore</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
+          <t>BF-FX</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Electricity_H2</t>
+          <t>iron</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>input</t>
+          <t>output</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6.508636363636362</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>fuel</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.6</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
+          <t>BOF-FX</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Iron ore_H2</t>
+          <t>iron</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1388,88 +1509,80 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.414285714285714</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>feedstock</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G20" t="n">
         <v>1</v>
       </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
+          <t>BOF-FX</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Scrap_H2</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>input</t>
+          <t>output</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.1571428571428571</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>feedstock</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H21" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
+          <t>H2-DRI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>Hydrogen_H2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>output</t>
+          <t>input</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="b">
-        <v>1</v>
-      </c>
+        <v>9.395454545454545</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>fuel</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>EAF</t>
+          <t>H2-DRI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Electricity_EAF</t>
+          <t>Electricity_H2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1478,7 +1591,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>6.508636363636362</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1486,22 +1599,22 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G23" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EAF</t>
+          <t>H2-DRI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Hydrogen_EAF</t>
+          <t>Iron ore_H2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1510,62 +1623,54 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>1.414285714285714</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>fuel</t>
+          <t>feed_ore</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="G24" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>EAF</t>
+          <t>H2-DRI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Scrap_EAF</t>
+          <t>iron</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>input</t>
+          <t>output</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>feedstock</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G25" t="n">
         <v>1</v>
       </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>EAF</t>
+          <t>ESF</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HBI_EAF</t>
+          <t>iron</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1574,44 +1679,222 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.525</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>feedstock</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G26" t="n">
         <v>1</v>
       </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>ESF</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Scrap_H2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.1571428571428571</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>feed_scrap</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ESF</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>EAF</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Electricity_EAF</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>fuel</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Hydrogen_EAF</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>fuel</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Scrap_EAF</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>feed_scrap</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HBI_EAF</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>feed_scrap</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>steel</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>output</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D33" t="n">
         <v>1</v>
       </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="b">
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1626,402 +1909,245 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>process_id</t>
+          <t>from_process</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>company</t>
+          <t>to_process</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>baseline_technology</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>capacity</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>introduced_year</t>
+          <t>commodity_id</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pohang BF3</t>
+          <t>Pohang BF3 · iron</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>Pohang BF3 · steel</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4128000</v>
-      </c>
-      <c r="E2" t="n">
-        <v>2017</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HyundaiBF3</t>
+          <t>HyundaiBF3 · iron</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hyundai Steel</t>
+          <t>HyundaiBF3 · steel</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2013</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pohang BF4</t>
+          <t>Pohang BF4 · iron</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>Pohang BF4 · steel</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>3804000</v>
-      </c>
-      <c r="E4" t="n">
-        <v>2024</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gwangyang BF2</t>
+          <t>Gwangyang BF2 · iron</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>Gwangyang BF2 · steel</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>3239000</v>
-      </c>
-      <c r="E5" t="n">
-        <v>2006</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gwangyang BF1</t>
+          <t>Gwangyang BF1 · iron</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>Gwangyang BF1 · steel</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1683000</v>
-      </c>
-      <c r="E6" t="n">
-        <v>2013</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gwangyang BF5</t>
+          <t>Gwangyang BF5 · iron</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>Gwangyang BF5 · steel</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>4722000</v>
-      </c>
-      <c r="E7" t="n">
-        <v>2016</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HyundaiBF2</t>
+          <t>HyundaiBF2 · iron</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hyundai Steel</t>
+          <t>HyundaiBF2 · steel</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>4237000</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2010</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gwangyang BF4</t>
+          <t>Gwangyang BF4 · iron</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>Gwangyang BF4 · steel</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="E9" t="n">
-        <v>2022</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Gwangyang BF3</t>
+          <t>Gwangyang BF3 · iron</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>Gwangyang BF3 · steel</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>3624000</v>
-      </c>
-      <c r="E10" t="n">
-        <v>2020</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HyundaiBF1</t>
+          <t>HyundaiBF1 · iron</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hyundai Steel</t>
+          <t>HyundaiBF1 · steel</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>4127000</v>
-      </c>
-      <c r="E11" t="n">
-        <v>2010</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Pohang BF2</t>
+          <t>Pohang BF2 · iron</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>Pohang BF2 · steel</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="E12" t="n">
-        <v>2015</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Pohang FNX3</t>
+          <t>Pohang FNX3 · iron</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>Pohang FNX3 · steel</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>1914000</v>
-      </c>
-      <c r="E13" t="n">
-        <v>2015</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Pohang FNX2</t>
+          <t>Pohang FNX2 · iron</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>Pohang FNX2 · steel</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>1280000</v>
-      </c>
-      <c r="E14" t="n">
-        <v>2015</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>EAF1</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>EAF</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="E15" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>EAF2</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>EAF</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="E16" t="n">
-        <v>2027</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>EAF3</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>POSCO</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>EAF</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="E17" t="n">
-        <v>2029</v>
+          <t>iron</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2035,245 +2161,851 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>process_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>baseline_technology</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>company</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>commodity_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>capacity</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>introduced_year</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Pohang BF3 · iron</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>POSCO</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D2" t="n">
-        <v>32394000</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>4128000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2017</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Pohang BF3 · steel</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>POSCO</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D3" t="n">
-        <v>34051447</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>4128000</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2017</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>HyundaiBF3 · iron</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D4" t="n">
-        <v>34051447</v>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Hyundai Steel</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2013</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>POSCO</t>
+          <t>HyundaiBF3 · steel</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D5" t="n">
-        <v>34051447</v>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hyundai Steel</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2013</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Pohang BF4 · iron</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>POSCO</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D6" t="n">
-        <v>34051447</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>3804000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Pohang BF4 · steel</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>POSCO</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D7" t="n">
-        <v>34051447</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>3804000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hyundai Steel</t>
+          <t>Gwangyang BF2 · iron</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D8" t="n">
-        <v>12364000</v>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3239000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2006</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hyundai Steel</t>
+          <t>Gwangyang BF2 · steel</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>2030</v>
-      </c>
-      <c r="D9" t="n">
-        <v>10706553</v>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>3239000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2006</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Hyundai Steel</t>
+          <t>Gwangyang BF1 · iron</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>2035</v>
-      </c>
-      <c r="D10" t="n">
-        <v>10706553</v>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1683000</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2013</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hyundai Steel</t>
+          <t>Gwangyang BF1 · steel</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D11" t="n">
-        <v>10706553</v>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1683000</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2013</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Hyundai Steel</t>
+          <t>Gwangyang BF5 · iron</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>2045</v>
-      </c>
-      <c r="D12" t="n">
-        <v>10706553</v>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>4722000</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2016</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Gwangyang BF5 · steel</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>4722000</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HyundaiBF2 · iron</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>Hyundai Steel</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>steel</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>2050</v>
-      </c>
-      <c r="D13" t="n">
-        <v>10706553</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>4237000</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HyundaiBF2 · steel</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Hyundai Steel</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>4237000</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Gwangyang BF4 · iron</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Gwangyang BF4 · steel</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Gwangyang BF3 · iron</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>3624000</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Gwangyang BF3 · steel</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>3624000</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>HyundaiBF1 · iron</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Hyundai Steel</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>4127000</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>HyundaiBF1 · steel</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Hyundai Steel</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>4127000</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Pohang BF2 · iron</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Pohang BF2 · steel</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Pohang FNX3 · iron</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BF-FX</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1914000</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Pohang FNX3 · steel</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BOF-FX</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1914000</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Pohang FNX2 · iron</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BF-FX</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1280000</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Pohang FNX2 · steel</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>BOF-FX</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1280000</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>EAF1 · steel</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>EAF2 · steel</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>EAF3 · steel</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>POSCO</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Korea steel</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2029</v>
       </c>
     </row>
   </sheetData>
@@ -2287,209 +3019,245 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>from_technology</t>
+          <t>company</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>to_technology</t>
+          <t>commodity_id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>action</t>
+          <t>year</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>capex_per_capacity</t>
+          <t>amount</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>replace</t>
-        </is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2025</v>
       </c>
       <c r="D2" t="n">
-        <v>425595</v>
+        <v>32394000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>replace</t>
-        </is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2030</v>
       </c>
       <c r="D3" t="n">
-        <v>1100000</v>
+        <v>34051447</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EAF</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>replace</t>
-        </is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2035</v>
       </c>
       <c r="D4" t="n">
-        <v>240000</v>
+        <v>34051447</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>replace</t>
-        </is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2040</v>
       </c>
       <c r="D5" t="n">
-        <v>500700</v>
+        <v>34051447</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>replace</t>
-        </is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2045</v>
       </c>
       <c r="D6" t="n">
-        <v>1100000</v>
+        <v>34051447</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>POSCO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EAF</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>replace</t>
-        </is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2050</v>
       </c>
       <c r="D7" t="n">
-        <v>240000</v>
+        <v>34051447</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EAF</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>replace</t>
-        </is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2025</v>
       </c>
       <c r="D8" t="n">
-        <v>500700</v>
+        <v>12364000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EAF</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>replace</t>
-        </is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2030</v>
       </c>
       <c r="D9" t="n">
-        <v>425595</v>
+        <v>10706553</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>EAF</t>
+          <t>Hyundai Steel</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>replace</t>
-        </is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2035</v>
       </c>
       <c r="D10" t="n">
-        <v>1100000</v>
+        <v>10706553</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Hyundai Steel</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2040</v>
+      </c>
+      <c r="D11" t="n">
+        <v>10706553</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Hyundai Steel</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2045</v>
+      </c>
+      <c r="D12" t="n">
+        <v>10706553</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Hyundai Steel</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>steel</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2050</v>
+      </c>
+      <c r="D13" t="n">
+        <v>10706553</v>
       </c>
     </row>
   </sheetData>
@@ -2498,6 +3266,162 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>from_technology</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>to_technology</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>capex_per_capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>H2-DRI</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>replace</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1100000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BF-FX</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>H2-DRI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>replace</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1100000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ESF</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>replace</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>330000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BOF-FX</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ESF</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>replace</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>330000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BOF</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>replace</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>240000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BOF-FX</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>replace</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>240000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2767,7 +3691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2790,12 +3714,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>iron</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>product</t>
+          <t>material</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2807,24 +3731,24 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BF gas_BB</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>product</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GJ</t>
+          <t>t</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BF gas_BX</t>
+          <t>BF gas_BB</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2841,7 +3765,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BOF gas_BB</t>
+          <t>BF gas_BX</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2858,7 +3782,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BOF gas_BB_2030</t>
+          <t>BOF gas_BB</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2875,7 +3799,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BOF gas_BX</t>
+          <t>BOF gas_BB_2030</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2892,7 +3816,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>COG_BB</t>
+          <t>BOF gas_BX</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2909,7 +3833,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>COG_BB_2030</t>
+          <t>COG_BB</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2926,7 +3850,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Coal_BB</t>
+          <t>COG_BB_2030</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2943,7 +3867,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Coal_BX</t>
+          <t>Coal_BB</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2960,7 +3884,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Electricity_EAF</t>
+          <t>Coal_BX</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2977,7 +3901,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Electricity_H2</t>
+          <t>Electricity_EAF</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2994,7 +3918,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Hydrogen_EAF</t>
+          <t>Electricity_H2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3011,7 +3935,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Hydrogen_H2</t>
+          <t>Hydrogen_EAF</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3028,7 +3952,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Natural gas_BX</t>
+          <t>Hydrogen_H2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3045,24 +3969,24 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HBI_BB</t>
+          <t>Natural gas_BX</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>material</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>GJ</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HBI_EAF</t>
+          <t>HBI_BB</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3079,7 +4003,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Iron ore_BB</t>
+          <t>HBI_EAF</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3096,7 +4020,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Iron ore_BX</t>
+          <t>Iron ore_BB</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3113,7 +4037,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Iron ore_H2</t>
+          <t>Iron ore_BX</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3130,7 +4054,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Scrap_BB</t>
+          <t>Iron ore_H2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3147,7 +4071,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Scrap_EAF</t>
+          <t>Scrap_BB</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3164,15 +4088,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Scrap_EAF</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>t</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Scrap_H2</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>material</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>t</t>
         </is>
@@ -4219,7 +5160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4242,7 +5183,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -4257,7 +5198,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>BOF</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -4265,14 +5206,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>renew, continue</t>
+          <t>replace, renew, continue</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
+          <t>BF-FX</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -4280,20 +5221,65 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>replace, renew, continue</t>
+          <t>renew, continue</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EAF</t>
+          <t>BOF-FX</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>20</v>
       </c>
       <c r="C5" t="inlineStr">
+        <is>
+          <t>renew, continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>H2-DRI</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>replace, renew, continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ESF</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>replace, renew, continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>replace, renew, continue</t>
         </is>
@@ -4310,7 +5296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4321,20 +5307,35 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>BF-BOF</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>BF-BOF-FX</t>
+          <t>BOF</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>H2-DRI-ESF</t>
+          <t>BF-FX</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
+        <is>
+          <t>BOF-FX</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>H2-DRI</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ESF</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>EAF</t>
         </is>
@@ -4348,12 +5349,21 @@
         <v>500700</v>
       </c>
       <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
         <v>425595</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
         <v>1100000</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
         <v>240000</v>
       </c>
     </row>
@@ -4365,12 +5375,21 @@
         <v>500700</v>
       </c>
       <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
         <v>425595</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
         <v>1100000</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
         <v>240000</v>
       </c>
     </row>
@@ -4382,12 +5401,21 @@
         <v>500700</v>
       </c>
       <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
         <v>425595</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
         <v>1100000</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
         <v>240000</v>
       </c>
     </row>
@@ -4399,12 +5427,21 @@
         <v>500700</v>
       </c>
       <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
         <v>425595</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
         <v>1100000</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
         <v>240000</v>
       </c>
     </row>
@@ -4416,12 +5453,21 @@
         <v>500700</v>
       </c>
       <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
         <v>425595</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
         <v>1100000</v>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
         <v>240000</v>
       </c>
     </row>
@@ -4433,12 +5479,21 @@
         <v>500700</v>
       </c>
       <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
         <v>425595</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
         <v>1100000</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>240000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(library): extract steel/shipping/petrochemical templates + fix steel blend data (L3a)
build_library.py extracts facility archetypes (one per baseline recipe, with
its transition alternatives and median capacity) and a flow-ordered chain from
each example workbook into the library; refreshes the index. Petrochemical
keeps the cracker/BTX trains (utility archetypes excluded).

Fixes a real data bug the new share-bound validation caught in steel.xlsx:
feed groups carried 'share of total charge' numbers under 'share of group sum'
semantics (BF/ESF single-member groups, BOF scrap+HBI Σmax=0.6<1), silently
forcing 2 demand-slack rows behind an 'optimal' status. Dropping the degenerate
groups and freeing the in-group scrap↔HBI mix cuts the objective 67x
(3.60e16 → 5.35e14) with ZERO unmet demand.

Library now ships 27 facilities across 4 sectors; all chains solve optimal.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/pathwise/public/examples/steel.xlsx
+++ b/frontend/pathwise/public/examples/steel.xlsx
@@ -1157,17 +1157,9 @@
       <c r="D8" t="n">
         <v>1.485</v>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>feed_ore</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.95</v>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1246,7 +1238,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="H11" t="inlineStr"/>
     </row>
@@ -1278,7 +1270,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="H12" t="inlineStr"/>
     </row>
@@ -1304,7 +1296,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="b">
+      <c r="H13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1455,17 +1447,9 @@
       <c r="D18" t="n">
         <v>1.65</v>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>feed_ore</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" t="n">
-        <v>1</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1538,7 +1522,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="b">
+      <c r="H21" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1625,17 +1609,9 @@
       <c r="D24" t="n">
         <v>1.414285714285714</v>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>feed_ore</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G24" t="n">
-        <v>1</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1705,17 +1681,9 @@
       <c r="D27" t="n">
         <v>0.1571428571428571</v>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>feed_scrap</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0.3</v>
-      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1740,7 +1708,7 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="b">
+      <c r="H28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1833,7 +1801,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
         <v>1</v>
@@ -1865,7 +1833,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
         <v>1</v>
@@ -1894,7 +1862,7 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="b">
+      <c r="H33" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>